<commit_message>
Update scanner fundamentals and portfolio
</commit_message>
<xml_diff>
--- a/output/NSE_Portfolio_Recommendations.xlsx
+++ b/output/NSE_Portfolio_Recommendations.xlsx
@@ -549,77 +549,77 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ARROWGREEN</t>
+          <t>SREEL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>814.1</v>
+        <v>279.4</v>
       </c>
       <c r="E2" t="n">
-        <v>548.8</v>
+        <v>209.71</v>
       </c>
       <c r="F2" t="n">
-        <v>48.34</v>
+        <v>33.23</v>
       </c>
       <c r="G2" t="n">
-        <v>659.2</v>
+        <v>241.57</v>
       </c>
       <c r="H2" t="n">
-        <v>23.5</v>
+        <v>15.66</v>
       </c>
       <c r="I2" t="n">
-        <v>67.94</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>1.35</v>
+        <v>2.4</v>
       </c>
       <c r="K2" t="n">
         <v>70</v>
       </c>
       <c r="L2" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>79.59999999999999</v>
+        <v>82</v>
       </c>
       <c r="N2" t="n">
-        <v>814.1</v>
+        <v>279.4</v>
       </c>
       <c r="O2" t="n">
-        <v>122</v>
+        <v>357</v>
       </c>
       <c r="P2" t="n">
         <v>100000</v>
       </c>
       <c r="Q2" t="n">
-        <v>99320.2</v>
+        <v>99745.8</v>
       </c>
       <c r="R2" t="n">
-        <v>9.93</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="S2" t="n">
-        <v>732.6900000000001</v>
+        <v>251.46</v>
       </c>
       <c r="T2" t="n">
-        <v>9932.02</v>
+        <v>9974.58</v>
       </c>
       <c r="U2" t="n">
-        <v>968.78</v>
+        <v>329.69</v>
       </c>
       <c r="V2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="W2" t="n">
-        <v>18870.84</v>
+        <v>17954.24</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>MODERATE CONVICTION</t>
+          <t>HIGH CONVICTION</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -634,77 +634,77 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GNFC</t>
+          <t>CUB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>596.7</v>
+        <v>238.48</v>
       </c>
       <c r="E3" t="n">
-        <v>493.23</v>
+        <v>205.82</v>
       </c>
       <c r="F3" t="n">
-        <v>20.98</v>
+        <v>15.87</v>
       </c>
       <c r="G3" t="n">
-        <v>539</v>
+        <v>245.38</v>
       </c>
       <c r="H3" t="n">
-        <v>10.71</v>
+        <v>-2.81</v>
       </c>
       <c r="I3" t="n">
-        <v>65.02</v>
+        <v>63.09</v>
       </c>
       <c r="J3" t="n">
-        <v>1.25</v>
+        <v>2.37</v>
       </c>
       <c r="K3" t="n">
         <v>70</v>
       </c>
       <c r="L3" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="M3" t="n">
-        <v>79.59999999999999</v>
+        <v>82</v>
       </c>
       <c r="N3" t="n">
-        <v>596.7</v>
+        <v>238.48</v>
       </c>
       <c r="O3" t="n">
-        <v>167</v>
+        <v>419</v>
       </c>
       <c r="P3" t="n">
         <v>100000</v>
       </c>
       <c r="Q3" t="n">
-        <v>99648.89999999999</v>
+        <v>99923.12</v>
       </c>
       <c r="R3" t="n">
-        <v>9.960000000000001</v>
+        <v>9.99</v>
       </c>
       <c r="S3" t="n">
-        <v>537.03</v>
+        <v>214.63</v>
       </c>
       <c r="T3" t="n">
-        <v>9964.889999999999</v>
+        <v>9992.309999999999</v>
       </c>
       <c r="U3" t="n">
-        <v>710.0700000000001</v>
+        <v>286.18</v>
       </c>
       <c r="V3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W3" t="n">
-        <v>18933.29</v>
+        <v>19984.62</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>MODERATE CONVICTION</t>
+          <t>HIGH CONVICTION</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -719,77 +719,77 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ANTELOPUS</t>
+          <t>GNFC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>957.15</v>
+        <v>597.9</v>
       </c>
       <c r="E4" t="n">
-        <v>644.87</v>
+        <v>493.76</v>
       </c>
       <c r="F4" t="n">
-        <v>48.43</v>
+        <v>21.09</v>
       </c>
       <c r="G4" t="n">
-        <v>720</v>
+        <v>539</v>
       </c>
       <c r="H4" t="n">
-        <v>32.94</v>
+        <v>10.93</v>
       </c>
       <c r="I4" t="n">
-        <v>64.95</v>
+        <v>65.45</v>
       </c>
       <c r="J4" t="n">
-        <v>2.51</v>
+        <v>1.87</v>
       </c>
       <c r="K4" t="n">
-        <v>75</v>
+        <v>72.5</v>
       </c>
       <c r="L4" t="n">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="M4" t="n">
-        <v>78.59999999999999</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>957.15</v>
+        <v>597.9</v>
       </c>
       <c r="O4" t="n">
-        <v>104</v>
+        <v>167</v>
       </c>
       <c r="P4" t="n">
         <v>100000</v>
       </c>
       <c r="Q4" t="n">
-        <v>99543.60000000001</v>
+        <v>99849.3</v>
       </c>
       <c r="R4" t="n">
-        <v>9.949999999999999</v>
+        <v>9.98</v>
       </c>
       <c r="S4" t="n">
-        <v>861.4400000000001</v>
+        <v>538.11</v>
       </c>
       <c r="T4" t="n">
-        <v>9954.360000000001</v>
+        <v>9984.93</v>
       </c>
       <c r="U4" t="n">
-        <v>1158.15</v>
+        <v>723.46</v>
       </c>
       <c r="V4" t="n">
         <v>21</v>
       </c>
       <c r="W4" t="n">
-        <v>20904.16</v>
+        <v>20968.35</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>MODERATE CONVICTION</t>
+          <t>HIGH CONVICTION</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -804,73 +804,73 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DICIND</t>
+          <t>KTKBANK</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>618.6</v>
+        <v>333.6</v>
       </c>
       <c r="E5" t="n">
-        <v>520.8099999999999</v>
+        <v>244.63</v>
       </c>
       <c r="F5" t="n">
-        <v>18.78</v>
+        <v>36.37</v>
       </c>
       <c r="G5" t="n">
-        <v>570</v>
+        <v>220.4</v>
       </c>
       <c r="H5" t="n">
-        <v>8.529999999999999</v>
+        <v>51.36</v>
       </c>
       <c r="I5" t="n">
-        <v>64.95999999999999</v>
+        <v>60.89</v>
       </c>
       <c r="J5" t="n">
-        <v>1.9</v>
+        <v>0.39</v>
       </c>
       <c r="K5" t="n">
-        <v>72.5</v>
+        <v>61.25</v>
       </c>
       <c r="L5" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="M5" t="n">
-        <v>77.5</v>
+        <v>76.75</v>
       </c>
       <c r="N5" t="n">
-        <v>618.6</v>
+        <v>333.6</v>
       </c>
       <c r="O5" t="n">
-        <v>161</v>
+        <v>299</v>
       </c>
       <c r="P5" t="n">
         <v>100000</v>
       </c>
       <c r="Q5" t="n">
-        <v>99594.60000000001</v>
+        <v>99746.39999999999</v>
       </c>
       <c r="R5" t="n">
-        <v>9.960000000000001</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="S5" t="n">
-        <v>556.74</v>
+        <v>300.24</v>
       </c>
       <c r="T5" t="n">
-        <v>9959.459999999999</v>
+        <v>9974.639999999999</v>
       </c>
       <c r="U5" t="n">
-        <v>742.3200000000001</v>
+        <v>393.65</v>
       </c>
       <c r="V5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="W5" t="n">
-        <v>19918.92</v>
+        <v>17954.35</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -889,73 +889,73 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PCJEWELLER</t>
+          <t>MAHABANK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>11.86</v>
+        <v>85</v>
       </c>
       <c r="E6" t="n">
-        <v>9.609999999999999</v>
+        <v>73.14</v>
       </c>
       <c r="F6" t="n">
-        <v>23.41</v>
+        <v>16.21</v>
       </c>
       <c r="G6" t="n">
-        <v>11.38</v>
+        <v>58.79</v>
       </c>
       <c r="H6" t="n">
-        <v>4.22</v>
+        <v>44.58</v>
       </c>
       <c r="I6" t="n">
-        <v>68.65000000000001</v>
+        <v>58.4</v>
       </c>
       <c r="J6" t="n">
-        <v>3.15</v>
+        <v>0.74</v>
       </c>
       <c r="K6" t="n">
-        <v>75</v>
+        <v>61.25</v>
       </c>
       <c r="L6" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="M6" t="n">
-        <v>77</v>
+        <v>76.75</v>
       </c>
       <c r="N6" t="n">
-        <v>11.86</v>
+        <v>85</v>
       </c>
       <c r="O6" t="n">
-        <v>8431</v>
+        <v>1176</v>
       </c>
       <c r="P6" t="n">
         <v>100000</v>
       </c>
       <c r="Q6" t="n">
-        <v>99991.66</v>
+        <v>99960</v>
       </c>
       <c r="R6" t="n">
         <v>10</v>
       </c>
       <c r="S6" t="n">
-        <v>10.67</v>
+        <v>76.5</v>
       </c>
       <c r="T6" t="n">
-        <v>9999.17</v>
+        <v>9996</v>
       </c>
       <c r="U6" t="n">
-        <v>14.35</v>
+        <v>99.45</v>
       </c>
       <c r="V6" t="n">
-        <v>20.99</v>
+        <v>17</v>
       </c>
       <c r="W6" t="n">
-        <v>20988.25</v>
+        <v>16993.2</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -974,73 +974,73 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KTKBANK</t>
+          <t>ANTELOPUS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>340.1</v>
+        <v>985.3</v>
       </c>
       <c r="E7" t="n">
-        <v>243.84</v>
+        <v>647.29</v>
       </c>
       <c r="F7" t="n">
-        <v>39.48</v>
+        <v>52.22</v>
       </c>
       <c r="G7" t="n">
-        <v>220.4</v>
+        <v>720</v>
       </c>
       <c r="H7" t="n">
-        <v>54.31</v>
+        <v>36.85</v>
       </c>
       <c r="I7" t="n">
-        <v>67.16</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>0.67</v>
+        <v>1.39</v>
       </c>
       <c r="K7" t="n">
-        <v>61.25</v>
+        <v>70</v>
       </c>
       <c r="L7" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="M7" t="n">
-        <v>76.75</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="N7" t="n">
-        <v>340.1</v>
+        <v>985.3</v>
       </c>
       <c r="O7" t="n">
-        <v>294</v>
+        <v>101</v>
       </c>
       <c r="P7" t="n">
         <v>100000</v>
       </c>
       <c r="Q7" t="n">
-        <v>99989.39999999999</v>
+        <v>99515.3</v>
       </c>
       <c r="R7" t="n">
-        <v>10</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="S7" t="n">
-        <v>306.09</v>
+        <v>886.77</v>
       </c>
       <c r="T7" t="n">
-        <v>9998.940000000001</v>
+        <v>9951.530000000001</v>
       </c>
       <c r="U7" t="n">
-        <v>401.32</v>
+        <v>1172.51</v>
       </c>
       <c r="V7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W7" t="n">
-        <v>17998.09</v>
+        <v>18907.91</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -1059,73 +1059,73 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MAHABANK</t>
+          <t>IMPAL</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>85.95</v>
+        <v>1114.2</v>
       </c>
       <c r="E8" t="n">
-        <v>73.02</v>
+        <v>1054.95</v>
       </c>
       <c r="F8" t="n">
-        <v>17.71</v>
+        <v>5.62</v>
       </c>
       <c r="G8" t="n">
-        <v>58.79</v>
+        <v>1128.1</v>
       </c>
       <c r="H8" t="n">
-        <v>46.2</v>
+        <v>-1.23</v>
       </c>
       <c r="I8" t="n">
-        <v>62.05</v>
+        <v>53.31</v>
       </c>
       <c r="J8" t="n">
-        <v>0.84</v>
+        <v>2.85</v>
       </c>
       <c r="K8" t="n">
-        <v>61.25</v>
+        <v>68.75</v>
       </c>
       <c r="L8" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="M8" t="n">
-        <v>76.75</v>
+        <v>75.25</v>
       </c>
       <c r="N8" t="n">
-        <v>85.95</v>
+        <v>1114.2</v>
       </c>
       <c r="O8" t="n">
-        <v>1163</v>
+        <v>89</v>
       </c>
       <c r="P8" t="n">
         <v>100000</v>
       </c>
       <c r="Q8" t="n">
-        <v>99959.85000000001</v>
+        <v>99163.8</v>
       </c>
       <c r="R8" t="n">
-        <v>10</v>
+        <v>9.92</v>
       </c>
       <c r="S8" t="n">
-        <v>77.36</v>
+        <v>1002.78</v>
       </c>
       <c r="T8" t="n">
-        <v>9995.98</v>
+        <v>9916.379999999999</v>
       </c>
       <c r="U8" t="n">
-        <v>100.56</v>
+        <v>1292.47</v>
       </c>
       <c r="V8" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="W8" t="n">
-        <v>16993.17</v>
+        <v>15866.21</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -1149,68 +1149,68 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>62.81</v>
+        <v>62.17</v>
       </c>
       <c r="E9" t="n">
-        <v>49.72</v>
+        <v>49.73</v>
       </c>
       <c r="F9" t="n">
-        <v>26.32</v>
+        <v>25.02</v>
       </c>
       <c r="G9" t="n">
         <v>62.84</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.05</v>
+        <v>-1.07</v>
       </c>
       <c r="I9" t="n">
-        <v>75.44</v>
+        <v>72.87</v>
       </c>
       <c r="J9" t="n">
-        <v>3.16</v>
+        <v>1.06</v>
       </c>
       <c r="K9" t="n">
-        <v>60</v>
+        <v>58.75</v>
       </c>
       <c r="L9" t="n">
         <v>100</v>
       </c>
       <c r="M9" t="n">
-        <v>76</v>
+        <v>75.25</v>
       </c>
       <c r="N9" t="n">
-        <v>62.81</v>
+        <v>62.17</v>
       </c>
       <c r="O9" t="n">
-        <v>1592</v>
+        <v>1608</v>
       </c>
       <c r="P9" t="n">
         <v>100000</v>
       </c>
       <c r="Q9" t="n">
-        <v>99993.52</v>
+        <v>99969.36</v>
       </c>
       <c r="R9" t="n">
         <v>10</v>
       </c>
       <c r="S9" t="n">
-        <v>56.53</v>
+        <v>55.95</v>
       </c>
       <c r="T9" t="n">
-        <v>9999.35</v>
+        <v>9996.940000000001</v>
       </c>
       <c r="U9" t="n">
-        <v>72.86</v>
+        <v>71.5</v>
       </c>
       <c r="V9" t="n">
-        <v>16</v>
+        <v>15.01</v>
       </c>
       <c r="W9" t="n">
-        <v>15998.96</v>
+        <v>15005.4</v>
       </c>
       <c r="X9" t="inlineStr">
         <is>
@@ -1229,73 +1229,73 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JAYNECOIND</t>
+          <t>CPCAP</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>89.04000000000001</v>
+        <v>135.89</v>
       </c>
       <c r="E10" t="n">
-        <v>86.5</v>
+        <v>103.74</v>
       </c>
       <c r="F10" t="n">
-        <v>2.94</v>
+        <v>30.99</v>
       </c>
       <c r="G10" t="n">
-        <v>53</v>
+        <v>133.9</v>
       </c>
       <c r="H10" t="n">
-        <v>68</v>
+        <v>1.49</v>
       </c>
       <c r="I10" t="n">
-        <v>40.78</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>7.28</v>
+        <v>2.46</v>
       </c>
       <c r="K10" t="n">
-        <v>81.25</v>
+        <v>75</v>
       </c>
       <c r="L10" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="M10" t="n">
-        <v>75.95</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>89.04000000000001</v>
+        <v>135.89</v>
       </c>
       <c r="O10" t="n">
-        <v>1123</v>
+        <v>735</v>
       </c>
       <c r="P10" t="n">
         <v>100000</v>
       </c>
       <c r="Q10" t="n">
-        <v>99991.92</v>
+        <v>99879.14999999999</v>
       </c>
       <c r="R10" t="n">
-        <v>10</v>
+        <v>9.99</v>
       </c>
       <c r="S10" t="n">
-        <v>80.14</v>
+        <v>122.3</v>
       </c>
       <c r="T10" t="n">
-        <v>9999.190000000001</v>
+        <v>9987.92</v>
       </c>
       <c r="U10" t="n">
-        <v>107.74</v>
+        <v>161.71</v>
       </c>
       <c r="V10" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="W10" t="n">
-        <v>20998.3</v>
+        <v>18977.04</v>
       </c>
       <c r="X10" t="inlineStr">
         <is>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>STRONG RETEST</t>
+          <t>NOT A RECOVERY</t>
         </is>
       </c>
     </row>
@@ -1314,73 +1314,73 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CUB</t>
+          <t>ARROWGREEN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>236.01</v>
+        <v>805.1</v>
       </c>
       <c r="E11" t="n">
-        <v>205.62</v>
+        <v>550</v>
       </c>
       <c r="F11" t="n">
-        <v>14.78</v>
+        <v>46.38</v>
       </c>
       <c r="G11" t="n">
-        <v>245.38</v>
+        <v>659.2</v>
       </c>
       <c r="H11" t="n">
-        <v>-3.82</v>
+        <v>22.13</v>
       </c>
       <c r="I11" t="n">
-        <v>61.53</v>
+        <v>65.43000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>1.01</v>
+        <v>0.64</v>
       </c>
       <c r="K11" t="n">
-        <v>58.75</v>
+        <v>61.25</v>
       </c>
       <c r="L11" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="M11" t="n">
-        <v>75.25</v>
+        <v>74.34999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>236.01</v>
+        <v>805.1</v>
       </c>
       <c r="O11" t="n">
-        <v>423</v>
+        <v>124</v>
       </c>
       <c r="P11" t="n">
         <v>100000</v>
       </c>
       <c r="Q11" t="n">
-        <v>99832.23</v>
+        <v>99832.39999999999</v>
       </c>
       <c r="R11" t="n">
         <v>9.98</v>
       </c>
       <c r="S11" t="n">
-        <v>212.41</v>
+        <v>724.59</v>
       </c>
       <c r="T11" t="n">
-        <v>9983.219999999999</v>
+        <v>9983.24</v>
       </c>
       <c r="U11" t="n">
-        <v>276.13</v>
+        <v>950.02</v>
       </c>
       <c r="V11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W11" t="n">
-        <v>16971.48</v>
+        <v>17969.83</v>
       </c>
       <c r="X11" t="inlineStr">
         <is>

</xml_diff>